<commit_message>
start to work on combine templates
</commit_message>
<xml_diff>
--- a/empty_templates/East Midlands.xlsx
+++ b/empty_templates/East Midlands.xlsx
@@ -1615,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.140625" customWidth="1"/>
@@ -1688,6 +1688,9 @@
           <t>CHESTERFIELD ROYAL HOSPITAL NHS FOUNDATION TRUST</t>
         </is>
       </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1700,6 +1703,9 @@
           <t>KETTERING GENERAL HOSPITAL NHS FOUNDATION TRUST</t>
         </is>
       </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1712,6 +1718,9 @@
           <t>NORTHAMPTON GENERAL HOSPITAL NHS TRUST</t>
         </is>
       </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1724,6 +1733,9 @@
           <t>NOTTINGHAM UNIVERSITY HOSPITALS NHS TRUST</t>
         </is>
       </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1736,6 +1748,9 @@
           <t>SHERWOOD FOREST HOSPITALS NHS FOUNDATION TRUST</t>
         </is>
       </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1748,6 +1763,9 @@
           <t>UNITED LINCOLNSHIRE HOSPITALS NHS TRUST</t>
         </is>
       </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1760,6 +1778,9 @@
           <t>UNIVERSITY HOSPITALS OF DERBY AND BURTON NHS FOUNDATION TRUST</t>
         </is>
       </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1771,6 +1792,129 @@
         <is>
           <t>UNIVERSITY HOSPITALS OF LEICESTER NHS TRUST</t>
         </is>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>NHS DERBY AND DERBYSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CHESTERFIELD ROYAL HOSPITAL NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NHS NORTHAMPTONSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>KETTERING GENERAL HOSPITAL NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NHS NORTHAMPTONSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NORTHAMPTON GENERAL HOSPITAL NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NHS NOTTINGHAM AND NOTTINGHAMSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>NOTTINGHAM UNIVERSITY HOSPITALS NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NHS NOTTINGHAM AND NOTTINGHAMSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SHERWOOD FOREST HOSPITALS NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>NHS LINCOLNSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>UNITED LINCOLNSHIRE HOSPITALS NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C15">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>NHS DERBY AND DERBYSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>UNIVERSITY HOSPITALS OF DERBY AND BURTON NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>NHS LEICESTER, LEICESTERSHIRE AND RUTLAND INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>UNIVERSITY HOSPITALS OF LEICESTER NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C17">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1826,7 +1970,9 @@
           <t>CHESTERFIELD ROYAL HOSPITAL NHS FOUNDATION TRUST</t>
         </is>
       </c>
-      <c r="C2" s="68"/>
+      <c r="C2" s="68">
+        <v>1</v>
+      </c>
       <c r="D2" s="69"/>
       <c r="E2" s="69"/>
       <c r="F2" s="69"/>
@@ -1843,7 +1989,9 @@
           <t>KETTERING GENERAL HOSPITAL NHS FOUNDATION TRUST</t>
         </is>
       </c>
-      <c r="C3" s="69"/>
+      <c r="C3" s="69">
+        <v>1</v>
+      </c>
       <c r="D3" s="69"/>
       <c r="E3" s="69"/>
       <c r="F3" s="69"/>
@@ -1860,7 +2008,9 @@
           <t>NORTHAMPTON GENERAL HOSPITAL NHS TRUST</t>
         </is>
       </c>
-      <c r="C4" s="69"/>
+      <c r="C4" s="69">
+        <v>1</v>
+      </c>
       <c r="D4" s="69"/>
       <c r="E4" s="69"/>
       <c r="F4" s="69"/>
@@ -1877,7 +2027,9 @@
           <t>NOTTINGHAM UNIVERSITY HOSPITALS NHS TRUST</t>
         </is>
       </c>
-      <c r="C5" s="69"/>
+      <c r="C5" s="69">
+        <v>1</v>
+      </c>
       <c r="D5" s="69"/>
       <c r="E5" s="69"/>
       <c r="F5" s="69"/>
@@ -1894,7 +2046,9 @@
           <t>SHERWOOD FOREST HOSPITALS NHS FOUNDATION TRUST</t>
         </is>
       </c>
-      <c r="C6" s="69"/>
+      <c r="C6" s="69">
+        <v>1</v>
+      </c>
       <c r="D6" s="70"/>
       <c r="E6" s="70"/>
       <c r="F6" s="70"/>
@@ -1915,7 +2069,9 @@
           <t>UNITED LINCOLNSHIRE HOSPITALS NHS TRUST</t>
         </is>
       </c>
-      <c r="C7" s="69"/>
+      <c r="C7" s="69">
+        <v>1</v>
+      </c>
       <c r="D7" s="69"/>
       <c r="E7" s="69"/>
       <c r="F7" s="69"/>
@@ -1932,7 +2088,9 @@
           <t>UNIVERSITY HOSPITALS OF DERBY AND BURTON NHS FOUNDATION TRUST</t>
         </is>
       </c>
-      <c r="C8" s="69"/>
+      <c r="C8" s="69">
+        <v>1</v>
+      </c>
       <c r="D8" s="69"/>
       <c r="E8" s="69"/>
       <c r="F8" s="69"/>
@@ -1949,79 +2107,161 @@
           <t>UNIVERSITY HOSPITALS OF LEICESTER NHS TRUST</t>
         </is>
       </c>
-      <c r="C9" s="69"/>
+      <c r="C9" s="69">
+        <v>1</v>
+      </c>
       <c r="D9" s="69"/>
       <c r="E9" s="69"/>
       <c r="F9" s="69"/>
       <c r="G9" s="69"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="69"/>
-      <c r="B10" s="69"/>
-      <c r="C10" s="69"/>
+      <c r="A10" s="69" t="inlineStr">
+        <is>
+          <t>NHS DERBY AND DERBYSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B10" s="69" t="inlineStr">
+        <is>
+          <t>CHESTERFIELD ROYAL HOSPITAL NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C10" s="69">
+        <v>4</v>
+      </c>
       <c r="D10" s="69"/>
       <c r="E10" s="69"/>
       <c r="F10" s="69"/>
       <c r="G10" s="69"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="69"/>
-      <c r="B11" s="69"/>
-      <c r="C11" s="69"/>
+      <c r="A11" s="69" t="inlineStr">
+        <is>
+          <t>NHS NORTHAMPTONSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B11" s="69" t="inlineStr">
+        <is>
+          <t>KETTERING GENERAL HOSPITAL NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C11" s="69">
+        <v>4</v>
+      </c>
       <c r="D11" s="69"/>
       <c r="E11" s="69"/>
       <c r="F11" s="69"/>
       <c r="G11" s="69"/>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="69"/>
-      <c r="B12" s="69"/>
-      <c r="C12" s="69"/>
+      <c r="A12" s="69" t="inlineStr">
+        <is>
+          <t>NHS NORTHAMPTONSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B12" s="69" t="inlineStr">
+        <is>
+          <t>NORTHAMPTON GENERAL HOSPITAL NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C12" s="69">
+        <v>4</v>
+      </c>
       <c r="D12" s="69"/>
       <c r="E12" s="69"/>
       <c r="F12" s="69"/>
       <c r="G12" s="69"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="69"/>
-      <c r="B13" s="69"/>
-      <c r="C13" s="69"/>
+      <c r="A13" s="69" t="inlineStr">
+        <is>
+          <t>NHS NOTTINGHAM AND NOTTINGHAMSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B13" s="69" t="inlineStr">
+        <is>
+          <t>NOTTINGHAM UNIVERSITY HOSPITALS NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C13" s="69">
+        <v>4</v>
+      </c>
       <c r="D13" s="69"/>
       <c r="E13" s="69"/>
       <c r="F13" s="69"/>
       <c r="G13" s="69"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="69"/>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69"/>
+      <c r="A14" s="69" t="inlineStr">
+        <is>
+          <t>NHS NOTTINGHAM AND NOTTINGHAMSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B14" s="69" t="inlineStr">
+        <is>
+          <t>SHERWOOD FOREST HOSPITALS NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C14" s="69">
+        <v>4</v>
+      </c>
       <c r="D14" s="69"/>
       <c r="E14" s="69"/>
       <c r="F14" s="69"/>
       <c r="G14" s="69"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="69"/>
-      <c r="B15" s="69"/>
-      <c r="C15" s="69"/>
+      <c r="A15" s="69" t="inlineStr">
+        <is>
+          <t>NHS LINCOLNSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B15" s="69" t="inlineStr">
+        <is>
+          <t>UNITED LINCOLNSHIRE HOSPITALS NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C15" s="69">
+        <v>4</v>
+      </c>
       <c r="D15" s="69"/>
       <c r="E15" s="69"/>
       <c r="F15" s="69"/>
       <c r="G15" s="69"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="69"/>
-      <c r="B16" s="69"/>
-      <c r="C16" s="69"/>
+      <c r="A16" s="69" t="inlineStr">
+        <is>
+          <t>NHS DERBY AND DERBYSHIRE INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B16" s="69" t="inlineStr">
+        <is>
+          <t>UNIVERSITY HOSPITALS OF DERBY AND BURTON NHS FOUNDATION TRUST</t>
+        </is>
+      </c>
+      <c r="C16" s="69">
+        <v>4</v>
+      </c>
       <c r="D16" s="69"/>
       <c r="E16" s="69"/>
       <c r="F16" s="69"/>
       <c r="G16" s="69"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="69"/>
-      <c r="B17" s="69"/>
-      <c r="C17" s="69"/>
+      <c r="A17" s="69" t="inlineStr">
+        <is>
+          <t>NHS LEICESTER, LEICESTERSHIRE AND RUTLAND INTEGRATED CARE BOARD</t>
+        </is>
+      </c>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>UNIVERSITY HOSPITALS OF LEICESTER NHS TRUST</t>
+        </is>
+      </c>
+      <c r="C17" s="69">
+        <v>4</v>
+      </c>
       <c r="D17" s="69"/>
       <c r="E17" s="69"/>
       <c r="F17" s="69"/>

</xml_diff>